<commit_message>
Fix CodeRabbit review comments on Chad boundary Excel generator
- Add 7 missing CARRE/POL locality names to FRENCH_NAMES and ARABIC_NAMES
- Use token-level matching ("CS" in parts) instead of substring ("CS" in code)
- Add os.makedirs before wb.save to ensure output directory exists
- Regenerate CHAD.xlsx with fixes applied
</commit_message>
<xml_diff>
--- a/PES-U/boundary_data/CHAD.xlsx
+++ b/PES-U/boundary_data/CHAD.xlsx
@@ -4579,7 +4579,11 @@
           <t>Carre 6 Pol 46</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>كاريه 6 بول 46</t>
+        </is>
+      </c>
       <c r="J90" t="n">
         <v>12.135696</v>
       </c>
@@ -4624,7 +4628,11 @@
           <t>Carre 8 Pol 51</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>كاريه 8 بول 51</t>
+        </is>
+      </c>
       <c r="J91" t="n">
         <v>12.132312</v>
       </c>
@@ -4669,7 +4677,11 @@
           <t>Carre 5 Pol 50</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>كاريه 5 بول 50</t>
+        </is>
+      </c>
       <c r="J92" t="n">
         <v>12.138778</v>
       </c>
@@ -4714,7 +4726,11 @@
           <t>Carre 6 Pol 47</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>كاريه 6 بول 47</t>
+        </is>
+      </c>
       <c r="J93" t="n">
         <v>12.134566</v>
       </c>
@@ -4759,7 +4775,11 @@
           <t>Carre 7 Pol 48</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>كاريه 7 بول 48</t>
+        </is>
+      </c>
       <c r="J94" t="n">
         <v>12.133679</v>
       </c>
@@ -4804,7 +4824,11 @@
           <t>Carre 8 Pol 52</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>كاريه 8 بول 52</t>
+        </is>
+      </c>
       <c r="J95" t="n">
         <v>12.13367</v>
       </c>
@@ -4849,7 +4873,11 @@
           <t>Carre 9 Pol 42</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>كاريه 9 بول 42</t>
+        </is>
+      </c>
       <c r="J96" t="n">
         <v>12.132971</v>
       </c>

</xml_diff>